<commit_message>
Atualiza foto da estação 1015693161 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -22912,7 +22912,11 @@
           <t xml:space="preserve">1800 2100 2500 </t>
         </is>
       </c>
-      <c r="L432" t="inlineStr"/>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\1015693161.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 684592398 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -33660,7 +33660,11 @@
           <t xml:space="preserve">700 850 1800 2100 2300 2500 3500 </t>
         </is>
       </c>
-      <c r="L638" t="inlineStr"/>
+      <c r="L638" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\684592398.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 1013251072 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -18852,7 +18852,11 @@
           <t xml:space="preserve">1800 2500 </t>
         </is>
       </c>
-      <c r="L354" t="inlineStr"/>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\1013251072.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 1013250890 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -18020,7 +18020,11 @@
           <t xml:space="preserve">1800 2500 3500 </t>
         </is>
       </c>
-      <c r="L338" t="inlineStr"/>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\1013250890.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 698058577 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -40592,7 +40592,11 @@
           <t xml:space="preserve">700 850 1800 2100 2300 2500 3500 </t>
         </is>
       </c>
-      <c r="L771" t="inlineStr"/>
+      <c r="L771" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\698058577.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="772">
       <c r="A772" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 687290520 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -35600,7 +35600,11 @@
           <t xml:space="preserve">700 850 1800 2100 2300 2500 3500 </t>
         </is>
       </c>
-      <c r="L675" t="inlineStr"/>
+      <c r="L675" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\687290520.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="676">
       <c r="A676" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 690990839 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -37320,7 +37320,11 @@
           <t xml:space="preserve">850 1800 2100 2300 2500 3500 </t>
         </is>
       </c>
-      <c r="L708" t="inlineStr"/>
+      <c r="L708" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\690990839.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="709">
       <c r="A709" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 4740580 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -27924,7 +27924,11 @@
           <t xml:space="preserve">700 850 1800 2100 2300 2500 3500 </t>
         </is>
       </c>
-      <c r="L528" t="inlineStr"/>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\4740580.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="529">
       <c r="A529" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 684136554 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -33048,7 +33048,11 @@
           <t xml:space="preserve">700 1800 2100 2500 3500 </t>
         </is>
       </c>
-      <c r="L626" t="inlineStr"/>
+      <c r="L626" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\684136554.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="627">
       <c r="A627" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 379988089 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -27556,7 +27556,11 @@
           <t xml:space="preserve">700 850 1800 2100 2500 3500 </t>
         </is>
       </c>
-      <c r="L521" t="inlineStr"/>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\379988089.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="522">
       <c r="A522" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 1017036311 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -44832,7 +44832,11 @@
           <t xml:space="preserve">700 2300 3500 </t>
         </is>
       </c>
-      <c r="L852" t="inlineStr"/>
+      <c r="L852" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\1017036311.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="853">
       <c r="A853" t="n">

</xml_diff>

<commit_message>
Atualiza foto da estação 1009312992 e rebuild do site
</commit_message>
<xml_diff>
--- a/ERBs_Mar26_goiania_preprocessed.xlsx
+++ b/ERBs_Mar26_goiania_preprocessed.xlsx
@@ -10780,7 +10780,11 @@
           <t xml:space="preserve">700 1800 2500 3500 </t>
         </is>
       </c>
-      <c r="L199" t="inlineStr"/>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>erb-watching\erb_photos\1009312992.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">

</xml_diff>